<commit_message>
Update MD use-cases spreadsheet with Aurora MySQL controls
</commit_message>
<xml_diff>
--- a/docs/MD_Usecases (6).xlsx
+++ b/docs/MD_Usecases (6).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ai\ecs-enterprise-backup-latest\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Desktop\ecs\pramaan-next\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98E4C273-1BF5-4B37-B082-8884E3BBE94E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AFA7B46-BCC3-46F6-8FB4-77C35192F79F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MD_Usecases" sheetId="3" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="83">
   <si>
     <t>Usecases</t>
   </si>
@@ -101,9 +101,6 @@
     <t>Cross-framework control mapping</t>
   </si>
   <si>
-    <t>AI-generated evidence summaries</t>
-  </si>
-  <si>
     <t>Evidence validation control</t>
   </si>
   <si>
@@ -119,9 +116,6 @@
     <t>Encryption validation, access control validation, vulnerability validation</t>
   </si>
   <si>
-    <t>AI-assisted audit preparation</t>
-  </si>
-  <si>
     <t>Audit readiness automation</t>
   </si>
   <si>
@@ -270,6 +264,15 @@
   </si>
   <si>
     <t>Common evidence querying -Pre defined query</t>
+  </si>
+  <si>
+    <t>Automated evidence summaries</t>
+  </si>
+  <si>
+    <t>Automated audit preparation</t>
+  </si>
+  <si>
+    <t>Automated - no manual intervention.</t>
   </si>
 </sst>
 </file>
@@ -625,17 +628,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E20"/>
-  <sheetFormatPr defaultColWidth="47.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:E22"/>
+  <sheetFormatPr defaultColWidth="47.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="33.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.88671875" customWidth="1"/>
-    <col min="3" max="3" width="32.33203125" customWidth="1"/>
-    <col min="4" max="4" width="35.88671875" customWidth="1"/>
-    <col min="5" max="5" width="51.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.90625" customWidth="1"/>
+    <col min="3" max="3" width="32.36328125" customWidth="1"/>
+    <col min="4" max="4" width="35.90625" customWidth="1"/>
+    <col min="5" max="5" width="51.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -649,10 +652,10 @@
         <v>21</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -660,16 +663,16 @@
         <v>16</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
@@ -677,16 +680,16 @@
         <v>16</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
@@ -697,13 +700,13 @@
         <v>22</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
@@ -711,31 +714,31 @@
         <v>16</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="58" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>16</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
@@ -746,13 +749,13 @@
         <v>23</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
@@ -763,30 +766,30 @@
         <v>24</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
-        <v>25</v>
+        <v>80</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>19</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>7</v>
       </c>
@@ -794,16 +797,16 @@
         <v>19</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>8</v>
       </c>
@@ -811,33 +814,33 @@
         <v>19</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>18</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>9</v>
       </c>
@@ -845,33 +848,33 @@
         <v>18</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>18</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>10</v>
       </c>
@@ -879,16 +882,16 @@
         <v>18</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>11</v>
       </c>
@@ -896,16 +899,16 @@
         <v>18</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>12</v>
       </c>
@@ -913,33 +916,33 @@
         <v>17</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
-        <v>31</v>
+        <v>81</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>13</v>
       </c>
@@ -947,16 +950,16 @@
         <v>17</v>
       </c>
       <c r="C19" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D19" s="2" t="s">
-        <v>35</v>
-      </c>
       <c r="E19" s="2" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>14</v>
       </c>
@@ -964,13 +967,18 @@
         <v>17</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>70</v>
+        <v>68</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D22" s="2" t="s">
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -982,633 +990,633 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H24"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="31.33203125" customWidth="1"/>
+    <col min="1" max="1" width="31.36328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>36</v>
-      </c>
       <c r="B3" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>22</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>23</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>24</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A12" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="H10" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="H11" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
+      <c r="B12" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="A13" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="A14" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="A15" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A13" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A14" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="H14" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A15" s="2" t="s">
-        <v>45</v>
-      </c>
       <c r="B15" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="A17" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="A18" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="G16" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="H16" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A17" s="2" t="s">
+      <c r="B18" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A19" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A20" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A21" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A22" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B17" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A18" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="G18" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="H18" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A19" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="G19" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="H19" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A20" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="G20" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="H20" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A21" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="G21" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="H21" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A22" s="2" t="s">
-        <v>32</v>
-      </c>
       <c r="B22" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>

</xml_diff>